<commit_message>
Fix question loader to read Column I for answers
</commit_message>
<xml_diff>
--- a/questions/question.xlsx
+++ b/questions/question.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\csryou\Desktop\quiz-project\questions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10980416-8A95-47EB-A610-D09EF77330B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F456702-1E97-4D7C-B8D2-59CC82B97AE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="11370" firstSheet="3" activeTab="4" xr2:uid="{C2D6912E-C08B-421F-A500-3E2A6D20402B}"/>
+    <workbookView xWindow="20" yWindow="380" windowWidth="19180" windowHeight="10900" firstSheet="3" activeTab="4" xr2:uid="{C2D6912E-C08B-421F-A500-3E2A6D20402B}"/>
   </bookViews>
   <sheets>
     <sheet name="easy" sheetId="1" r:id="rId1"/>
@@ -271,7 +271,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -296,11 +296,20 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="游ゴシック"/>
+      <family val="3"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="10"/>
       <color rgb="FF434343"/>
-      <name val="ＭＳ ゴシック"/>
+      <name val="游ゴシック"/>
       <family val="3"/>
       <charset val="128"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -325,7 +334,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -335,7 +344,13 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -913,7 +928,7 @@
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" t="s">
+      <c r="A2" s="4" t="s">
         <v>14</v>
       </c>
       <c r="B2" t="s">
@@ -931,13 +946,13 @@
       <c r="F2" t="s">
         <v>18</v>
       </c>
-      <c r="I2" t="str">
+      <c r="H2" t="str">
         <f>F2</f>
         <v>店の扉が開いた</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.55000000000000004">
-      <c r="A3" t="s">
+      <c r="A3" s="4" t="s">
         <v>19</v>
       </c>
       <c r="B3" t="s">
@@ -955,13 +970,13 @@
       <c r="F3" t="s">
         <v>22</v>
       </c>
-      <c r="I3" t="str">
+      <c r="H3" s="3" t="str">
         <f>F3</f>
         <v>膝が曲がっていて伸ばすと長い</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="5" t="s">
         <v>23</v>
       </c>
       <c r="B4" t="s">
@@ -979,7 +994,7 @@
       <c r="F4" t="s">
         <v>27</v>
       </c>
-      <c r="I4" t="str">
+      <c r="H4" t="str">
         <f>F4</f>
         <v>ガスト</v>
       </c>
@@ -987,5 +1002,6 @@
   </sheetData>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix formula parsing and add debug logs
</commit_message>
<xml_diff>
--- a/questions/question.xlsx
+++ b/questions/question.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\csryou\Desktop\quiz-project\questions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F456702-1E97-4D7C-B8D2-59CC82B97AE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C6B3398-8DD5-4AD3-BAE2-5BBB856F8CBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20" yWindow="380" windowWidth="19180" windowHeight="10900" firstSheet="3" activeTab="4" xr2:uid="{C2D6912E-C08B-421F-A500-3E2A6D20402B}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="11370" firstSheet="3" activeTab="4" xr2:uid="{C2D6912E-C08B-421F-A500-3E2A6D20402B}"/>
   </bookViews>
   <sheets>
     <sheet name="easy" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="33">
   <si>
     <t>問題</t>
     <rPh sb="0" eb="2">
@@ -264,6 +264,44 @@
   </si>
   <si>
     <t>ガスト</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>無線通信規格「Bluetooth」の語源となった王様はどこの国の人？</t>
+    <rPh sb="0" eb="4">
+      <t>ムセンツウシン</t>
+    </rPh>
+    <rPh sb="4" eb="6">
+      <t>キカク</t>
+    </rPh>
+    <rPh sb="18" eb="20">
+      <t>ゴゲン</t>
+    </rPh>
+    <rPh sb="24" eb="26">
+      <t>オウサマ</t>
+    </rPh>
+    <rPh sb="30" eb="31">
+      <t>クニ</t>
+    </rPh>
+    <rPh sb="32" eb="33">
+      <t>ヒト</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>デンマーク</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ロシア</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>フランス</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ブルガリア</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -334,7 +372,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -342,9 +380,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
@@ -890,7 +925,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{690150B6-791B-41CB-87CD-167041B46E25}">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="45.58203125" customWidth="1"/>
@@ -928,7 +963,7 @@
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B2" t="s">
@@ -952,7 +987,7 @@
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.55000000000000004">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="3" t="s">
         <v>19</v>
       </c>
       <c r="B3" t="s">
@@ -970,13 +1005,13 @@
       <c r="F3" t="s">
         <v>22</v>
       </c>
-      <c r="H3" s="3" t="str">
+      <c r="H3" t="str">
         <f>F3</f>
         <v>膝が曲がっていて伸ばすと長い</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="4" t="s">
         <v>23</v>
       </c>
       <c r="B4" t="s">
@@ -999,9 +1034,33 @@
         <v>ガスト</v>
       </c>
     </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="A5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" t="s">
+        <v>30</v>
+      </c>
+      <c r="E5" t="s">
+        <v>31</v>
+      </c>
+      <c r="F5" t="s">
+        <v>32</v>
+      </c>
+      <c r="H5" s="2" t="str">
+        <f>C5</f>
+        <v>デンマーク</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>